<commit_message>
Home: productos del cliente (38705, 38706, 38707, 38708, 38702, 38709) y skeleton de carga (38698)
- 38705 ahorro, 38707 prestamos, 38708 rotativo y 38702 pre-aprobado: automatizados y ejecutados con exito.

- 38706 corriente y 38709 saldos: construidos; pendientes de datos (cliente con cuenta corriente y montos del backend).

- 38698 skeleton: lectura de la pagina por DevTools del WebView (WebViewDevTools).

- Control: columnas TipoProducto y Monto; catalogo en orden alfabetico (20 casos).

- Listado: columna PRODUCTOS_HOME para elegir clientes por producto; clave rechazada queda FALLIDO.

- README y Consolidacion_Casos_de_Prueba (version 3, control de cambios) actualizados.
</commit_message>
<xml_diff>
--- a/datos/pool_clientes_plantilla.xlsx
+++ b/datos/pool_clientes_plantilla.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Clientes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Leyenda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clientes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leyenda" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Clientes'!$A$1:$H$69283</definedName>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -492,6 +492,11 @@
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>LINEA_SMS</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>PRODUCTOS_HOME</t>
         </is>
       </c>
     </row>

</xml_diff>